<commit_message>
added [M+H - O=C=NCH3 (methyl isocyanate)]+
</commit_message>
<xml_diff>
--- a/inst/extdata/CAMERA_rules_neg.xlsx
+++ b/inst/extdata/CAMERA_rules_neg.xlsx
@@ -8,10 +8,10 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tmh331\Desktop\gits\commonMZ\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF5AE91D-74E0-45DC-9E20-57E5539F6877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1FA738-28E2-4129-A620-3C2D7B87EDED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockWindows="1"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36915" yWindow="690" windowWidth="21600" windowHeight="12675" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="rules_jan_neg" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t>name</t>
   </si>
@@ -493,6 +493,9 @@
   </si>
   <si>
     <t>[M-H-H2O-acetyl]-</t>
+  </si>
+  <si>
+    <t>[M-H - O=C=NCH3 (methyl isocyanate)]-</t>
   </si>
 </sst>
 </file>
@@ -614,7 +617,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -630,6 +633,9 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -978,10 +984,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G147"/>
+  <dimension ref="A1:G148"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.85546875"/>
+    <col min="1" max="1" width="40.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -4395,6 +4401,30 @@
         <v>0</v>
       </c>
       <c r="G147" s="14">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A148" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="B148" s="14">
+        <v>1</v>
+      </c>
+      <c r="C148" s="14">
+        <v>1</v>
+      </c>
+      <c r="D148">
+        <f>-(57.02146-$D$2)</f>
+        <v>-58.028736455000001</v>
+      </c>
+      <c r="E148" s="14">
+        <v>182</v>
+      </c>
+      <c r="F148" s="14">
+        <v>0</v>
+      </c>
+      <c r="G148" s="14">
         <v>0.5</v>
       </c>
     </row>

</xml_diff>